<commit_message>
Yes there is significant changes than mentioned i# with '#' will be ignored, and an empty message aborts the commit.
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Desktop\Git1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C833B5D-B66A-4C5C-9EB7-96E5D8C58409}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FB758A-3B65-440F-A6DF-CD7D493A9F8D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,12 +25,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>sdfsfs</t>
   </si>
   <si>
     <t>sfsfsd</t>
+  </si>
+  <si>
+    <t>fsdfdsfs</t>
   </si>
 </sst>
 </file>
@@ -348,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D4:J4"/>
+  <dimension ref="D4:J12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="4" spans="4:10" x14ac:dyDescent="0.3">
@@ -359,6 +362,11 @@
         <v>1</v>
       </c>
     </row>
+    <row r="12" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="H12" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
New file checking file.txt added and test.xlsx modified
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Desktop\Git1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FB758A-3B65-440F-A6DF-CD7D493A9F8D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6963E8-9B79-4E2D-954C-B0FF72ACC97D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>sdfsfs</t>
   </si>
@@ -34,6 +34,9 @@
   </si>
   <si>
     <t>fsdfdsfs</t>
+  </si>
+  <si>
+    <t>sfsfsdf</t>
   </si>
 </sst>
 </file>
@@ -351,10 +354,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D4:J12"/>
+  <dimension ref="D4:P12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="4" spans="4:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D4" t="s">
         <v>0</v>
       </c>
@@ -362,7 +365,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="4:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="P7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="4:16" x14ac:dyDescent="0.3">
       <c r="H12" t="s">
         <v>2</v>
       </c>

</xml_diff>